<commit_message>
Remove Definition sheet in xpert workload summary report
</commit_message>
<xml_diff>
--- a/api/templates/pk_xpert_workload_summary_report/en.xlsx
+++ b/api/templates/pk_xpert_workload_summary_report/en.xlsx
@@ -3,12 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Wise" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="District Wise" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Definition" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deployment Wise'!$A$7:$F$8</definedName>
@@ -103,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t xml:space="preserve">Xpert Workload Summary Report</t>
   </si>
@@ -151,36 +150,6 @@
   </si>
   <si>
     <t>&lt;approvalStatus&gt;</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Meaning</t>
-  </si>
-  <si>
-    <t>Blank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use the last assay used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GxAlert Active/Inactive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inactive if site is Inactive on GxAlert</t>
-  </si>
-  <si>
-    <t>Months</t>
-  </si>
-  <si>
-    <t>Month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blanks are "0"</t>
   </si>
 </sst>
 </file>
@@ -1006,61 +975,4 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="23.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" width="53.5703125"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>